<commit_message>
feat: Add apresentação + Melhorar gráficos
- Adicionado apresentação powerpoint
- Corrigido gráficos para usar numeração e rótulos de valor
</commit_message>
<xml_diff>
--- a/M2-M3_Analise_Heuristicas.xlsx
+++ b/M2-M3_Analise_Heuristicas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Herick\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Herick\Desktop\Projects\teoria-computacao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E1E6598-3065-4616-B0F6-B7CDA32A732F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{005FAE58-F67D-4DDF-A280-5F7C23C36578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conclusoes" sheetId="1" r:id="rId1"/>
@@ -261,7 +261,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -271,6 +270,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -432,6 +432,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="#,##0" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -452,7 +453,7 @@
               </a:p>
             </c:txPr>
             <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
+            <c:showVal val="1"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
@@ -461,6 +462,11 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="rect">
+                    <a:avLst/>
+                  </a:prstGeom>
+                </c15:spPr>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -644,7 +650,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -825,7 +831,7 @@
               </a:p>
             </c:txPr>
             <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
+            <c:showVal val="1"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
@@ -834,6 +840,11 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="rect">
+                    <a:avLst/>
+                  </a:prstGeom>
+                </c15:spPr>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1017,7 +1028,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1178,6 +1189,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="#,##0" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -1198,7 +1210,7 @@
               </a:p>
             </c:txPr>
             <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
+            <c:showVal val="1"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
@@ -1207,6 +1219,11 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="rect">
+                    <a:avLst/>
+                  </a:prstGeom>
+                </c15:spPr>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1390,7 +1407,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1578,6 +1595,11 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="rect">
+                    <a:avLst/>
+                  </a:prstGeom>
+                </c15:spPr>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -1806,7 +1828,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1967,6 +1989,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="#,##0.00" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -1987,7 +2010,7 @@
               </a:p>
             </c:txPr>
             <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
+            <c:showVal val="1"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
@@ -1996,6 +2019,11 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="rect">
+                    <a:avLst/>
+                  </a:prstGeom>
+                </c15:spPr>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -2377,6 +2405,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="#,##0" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -2390,6 +2419,9 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="002060"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
@@ -2397,7 +2429,7 @@
               </a:p>
             </c:txPr>
             <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
+            <c:showVal val="1"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
@@ -2406,6 +2438,11 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="rect">
+                    <a:avLst/>
+                  </a:prstGeom>
+                </c15:spPr>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -2497,6 +2534,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="#,##0" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -2510,14 +2548,18 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="C00000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
                 <a:endParaRPr lang="pt-BR"/>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
+            <c:showVal val="1"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
@@ -2526,6 +2568,11 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="rect">
+                    <a:avLst/>
+                  </a:prstGeom>
+                </c15:spPr>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -2728,7 +2775,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2889,6 +2936,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="#,##0.00" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -2902,6 +2950,9 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="002060"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
@@ -2909,7 +2960,7 @@
               </a:p>
             </c:txPr>
             <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
+            <c:showVal val="1"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
@@ -2918,6 +2969,11 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="rect">
+                    <a:avLst/>
+                  </a:prstGeom>
+                </c15:spPr>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -2998,7 +3054,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="93A9CE"/>
+              <a:srgbClr val="C00000"/>
             </a:solidFill>
             <a:ln w="9360">
               <a:solidFill>
@@ -3009,6 +3065,138 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="1.3052549358163993E-2"/>
+                  <c:y val="0"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="1"/>
+              <c:separator> </c:separator>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-A30D-4979-8049-56ED45851105}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="1.1187899449854899E-2"/>
+                  <c:y val="0"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="1"/>
+              <c:separator> </c:separator>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-A30D-4979-8049-56ED45851105}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="1.1187899449854866E-2"/>
+                  <c:y val="0"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="1"/>
+              <c:separator> </c:separator>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-A30D-4979-8049-56ED45851105}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="9.3232495415457219E-3"/>
+                  <c:y val="0"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="1"/>
+              <c:separator> </c:separator>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-A30D-4979-8049-56ED45851105}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="1.1187899449854866E-2"/>
+                  <c:y val="-1.4372528111870567E-16"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="1"/>
+              <c:separator> </c:separator>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-A30D-4979-8049-56ED45851105}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="9.3232495415457219E-3"/>
+                  <c:y val="-1.4372528111870567E-16"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="1"/>
+              <c:separator> </c:separator>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-A30D-4979-8049-56ED45851105}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -3022,6 +3210,9 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" strike="noStrike" spc="-1">
+                    <a:solidFill>
+                      <a:srgbClr val="C00000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
@@ -3029,7 +3220,7 @@
               </a:p>
             </c:txPr>
             <c:showLegendKey val="0"/>
-            <c:showVal val="0"/>
+            <c:showVal val="1"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
@@ -3038,6 +3229,11 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="rect">
+                    <a:avLst/>
+                  </a:prstGeom>
+                </c15:spPr>
                 <c15:showLeaderLines val="1"/>
               </c:ext>
             </c:extLst>
@@ -3240,7 +3436,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3752,7 +3948,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3991,15 +4187,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>160560</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>614355</xdr:colOff>
-      <xdr:row>45</xdr:row>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>195255</xdr:colOff>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>182880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4104,16 +4300,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>46</xdr:row>
-      <xdr:rowOff>10080</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>555</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>10080</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>11520</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>86280</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>1995</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4327,87 +4523,87 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4"/>
+      <c r="A2" s="3"/>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4"/>
+      <c r="A6" s="3"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
+      <c r="A9" s="3"/>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
+      <c r="A14" s="3"/>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="4"/>
+      <c r="A17" s="3"/>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>13</v>
       </c>
     </row>
@@ -4433,28 +4629,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>21</v>
       </c>
     </row>
@@ -19897,124 +20093,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
     </row>
     <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="7">
         <f>AVERAGEIF(Dados!$A$2:$A$601,"primeiramelhora",Dados!$F$2:$F$601)</f>
         <v>53257.1</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="7">
         <f>_xlfn.MAXIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"primeiramelhora")</f>
         <v>412035</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="7">
         <f>AVERAGEIF(Dados!$A$2:$A$601,"primeiramelhora",Dados!$E$2:$E$601)</f>
         <v>9.6772833333333317</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="7">
         <f>_xlfn.MAXIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"primeiramelhora")</f>
         <v>76.495999999999995</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="7">
         <f>AVERAGEIF(Dados!$A$2:$A$601,"primeiramelhora",Dados!$G$2:$G$601)</f>
         <v>979.15</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="7">
         <f>AVERAGEIF(Dados!$A$2:$A$601,"monotonarandomizada",Dados!$F$2:$F$601)</f>
         <v>1943.2037037037037</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="7">
         <f>_xlfn.MAXIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada")</f>
         <v>5495</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="7">
         <f>AVERAGEIF(Dados!$A$2:$A$601,"monotonarandomizada",Dados!$E$2:$E$601)</f>
         <v>0.35362222222222228</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="7">
         <f>_xlfn.MAXIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada")</f>
         <v>1.3720000000000001</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="7">
         <f>AVERAGEIF(Dados!$A$2:$A$601,"monotonarandomizada",Dados!$G$2:$G$601)</f>
         <v>976.62777777777774</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,0.1)</f>
         <v>2242.5500000000002</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="7">
         <f>_xlfn.MAXIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,0.1)</f>
         <v>5495</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,0.1)</f>
         <v>0.40778333333333339</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="7">
         <f>_xlfn.MAXIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,0.1)</f>
         <v>1.3720000000000001</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,0.1)</f>
         <v>906.3</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A8:F8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -20034,187 +20229,187 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="7">
+      <c r="A4" s="6">
         <v>0.1</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A4)</f>
         <v>2242.5500000000002</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A4)</f>
         <v>0.40778333333333339</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A4)</f>
         <v>906.3</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="6">
         <v>0.2</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A5)</f>
         <v>2104.9333333333334</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A5)</f>
         <v>0.40294999999999986</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A5)</f>
         <v>933.05</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
+      <c r="A6" s="6">
         <v>0.3</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A6)</f>
         <v>1835.7666666666667</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A6)</f>
         <v>0.33109999999999995</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A6)</f>
         <v>964.65</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+      <c r="A7" s="6">
         <v>0.4</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A7)</f>
         <v>1860.6666666666667</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A7)</f>
         <v>0.3385999999999999</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A7)</f>
         <v>968.4</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
+      <c r="A8" s="6">
         <v>0.5</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A8)</f>
         <v>2015.5166666666667</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A8)</f>
         <v>0.37065000000000003</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A8)</f>
         <v>969.73333333333335</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
+      <c r="A9" s="6">
         <v>0.6</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A9)</f>
         <v>1944.3333333333333</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A9)</f>
         <v>0.35499999999999993</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A9)</f>
         <v>992.91666666666663</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="7">
+      <c r="A10" s="6">
         <v>0.7</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A10)</f>
         <v>1833.4166666666667</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A10)</f>
         <v>0.33123333333333327</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A10)</f>
         <v>1007.9</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="7">
+      <c r="A11" s="6">
         <v>0.8</v>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A11)</f>
         <v>1789.1</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A11)</f>
         <v>0.32050000000000001</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A11)</f>
         <v>1019.7166666666667</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="7">
+      <c r="A12" s="6">
         <v>0.9</v>
       </c>
-      <c r="B12" s="8">
+      <c r="B12" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A12)</f>
         <v>1862.55</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A12)</f>
         <v>0.32478333333333331</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$H$2:$H$601,A12)</f>
         <v>1026.9833333333333</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -20238,230 +20433,230 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
     </row>
     <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="7">
-        <v>10</v>
-      </c>
-      <c r="B4" s="7">
+      <c r="A4" s="6">
+        <v>10</v>
+      </c>
+      <c r="B4" s="6">
         <v>32</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A4,Dados!$B$2:$B$601,B4)</f>
         <v>171.5</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A4,Dados!$B$2:$B$601,B4,Dados!$H$2:$H$601,0.1)</f>
         <v>195</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A4,Dados!$B$2:$B$601,B4)</f>
         <v>6.0000000000000012E-2</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A4,Dados!$B$2:$B$601,B4,Dados!$H$2:$H$601,0.1)</f>
         <v>0.21669999999999998</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A4,Dados!$B$2:$B$601,B4)</f>
         <v>1004</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A4,Dados!$B$2:$B$601,B4,Dados!$H$2:$H$601,0.1)</f>
         <v>1807.4</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
-        <v>10</v>
-      </c>
-      <c r="B5" s="7">
+      <c r="A5" s="6">
+        <v>10</v>
+      </c>
+      <c r="B5" s="6">
         <v>100</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A5,Dados!$B$2:$B$601,B5)</f>
         <v>527.70000000000005</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A5,Dados!$B$2:$B$601,B5,Dados!$H$2:$H$601,0.1)</f>
         <v>533.29999999999995</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A5,Dados!$B$2:$B$601,B5)</f>
         <v>0.14679999999999999</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A5,Dados!$B$2:$B$601,B5,Dados!$H$2:$H$601,0.1)</f>
         <v>0.18959999999999999</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A5,Dados!$B$2:$B$601,B5)</f>
         <v>2717.8</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A5,Dados!$B$2:$B$601,B5,Dados!$H$2:$H$601,0.1)</f>
         <v>1768.9</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
+      <c r="A6" s="6">
         <v>20</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <v>89</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A6,Dados!$B$2:$B$601,B6)</f>
         <v>304.2</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A6,Dados!$B$2:$B$601,B6,Dados!$H$2:$H$601,0.1)</f>
         <v>294.5</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A6,Dados!$B$2:$B$601,B6)</f>
         <v>0.54859999999999998</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A6,Dados!$B$2:$B$601,B6,Dados!$H$2:$H$601,0.1)</f>
         <v>0.29299999999999998</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A6,Dados!$B$2:$B$601,B6)</f>
         <v>5514</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A6,Dados!$B$2:$B$601,B6,Dados!$H$2:$H$601,0.1)</f>
         <v>2067.1999999999998</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+      <c r="A7" s="6">
         <v>20</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="6">
         <v>400</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A7,Dados!$B$2:$B$601,B7)</f>
         <v>1253.5</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A7,Dados!$B$2:$B$601,B7,Dados!$H$2:$H$601,0.1)</f>
         <v>1092.0999999999999</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A7,Dados!$B$2:$B$601,B7)</f>
         <v>1.5487</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A7,Dados!$B$2:$B$601,B7,Dados!$H$2:$H$601,0.1)</f>
         <v>0.31179999999999997</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A7,Dados!$B$2:$B$601,B7)</f>
         <v>17036.2</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A7,Dados!$B$2:$B$601,B7,Dados!$H$2:$H$601,0.1)</f>
         <v>2021.1</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
+      <c r="A8" s="6">
         <v>50</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="6">
         <v>354</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A8,Dados!$B$2:$B$601,B8)</f>
         <v>583.29999999999995</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A8,Dados!$B$2:$B$601,B8,Dados!$H$2:$H$601,0.1)</f>
         <v>493.5</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A8,Dados!$B$2:$B$601,B8)</f>
         <v>8.5229999999999997</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A8,Dados!$B$2:$B$601,B8,Dados!$H$2:$H$601,0.1)</f>
         <v>0.52710000000000001</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A8,Dados!$B$2:$B$601,B8)</f>
         <v>43662.5</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A8,Dados!$B$2:$B$601,B8,Dados!$H$2:$H$601,0.1)</f>
         <v>2184.1999999999998</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
+      <c r="A9" s="6">
         <v>50</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="6">
         <v>2500</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A9,Dados!$B$2:$B$601,B9)</f>
         <v>3034.7</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="7">
         <f>AVERAGEIFS(Dados!$G$2:$G$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A9,Dados!$B$2:$B$601,B9,Dados!$H$2:$H$601,0.1)</f>
         <v>2829.4</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A9,Dados!$B$2:$B$601,B9)</f>
         <v>47.236599999999996</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="7">
         <f>AVERAGEIFS(Dados!$E$2:$E$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A9,Dados!$B$2:$B$601,B9,Dados!$H$2:$H$601,0.1)</f>
         <v>0.90849999999999986</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"primeiramelhora",Dados!$C$2:$C$601,A9,Dados!$B$2:$B$601,B9)</f>
         <v>249608.1</v>
       </c>
-      <c r="H9" s="8">
+      <c r="H9" s="7">
         <f>AVERAGEIFS(Dados!$F$2:$F$601,Dados!$A$2:$A$601,"monotonarandomizada",Dados!$C$2:$C$601,A9,Dados!$B$2:$B$601,B9,Dados!$H$2:$H$601,0.1)</f>
         <v>3606.5</v>
       </c>

</xml_diff>